<commit_message>
Update PR5 y PR6
</commit_message>
<xml_diff>
--- a/documentation/Construccion y Evolucion/2. Reportes de problemas/PR 5.xlsx
+++ b/documentation/Construccion y Evolucion/2. Reportes de problemas/PR 5.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\TraductorBraille\documentation\Construccion y Evolucion\2. Reportes de problemas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\EPN\SEXTO SEMESTRE\Construccion y evolucion software\traductor_braile_español\TraductorBrailleEspanol\documentation\Construccion y Evolucion\2. Reportes de problemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491B549D-318D-4725-98F8-208AD35D5E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{AAACD53E-982C-4521-B07F-7DC6290E23F5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="PR Formato" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="15">
   <si>
     <t>Reporte de Problema</t>
   </si>
@@ -64,13 +63,19 @@
   </si>
   <si>
     <t>No se ha logrado localizar la descripción del proyecto dentro de los documentos del sistema.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inexistencia de un documento dedicado a la descripción y visión del proyecto. Dentro del repositorio a pesar de la extensa documentación presente sobre el producto, se ignoró totalmente el echo de describir el problema inicial presentado por tomar por hecho que estaba estaba sobreentendido por todos los miembros del equipo. </t>
+  </si>
+  <si>
+    <t>Crear un archivo dentro del repositorio donde se exprese todo el contexto inicial del proyecto, desde el planteamiento del problema, requisitos generales, hasta lo que está fuera del alcance del poyecto.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,7 +321,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -333,53 +338,71 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -714,21 +737,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F84A08-0160-4953-9528-DB07A5F993CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:H28"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="5.5703125" customWidth="1"/>
-    <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5703125" customWidth="1"/>
-    <col min="5" max="7" width="20.140625" customWidth="1"/>
-    <col min="8" max="8" width="5.5703125" customWidth="1"/>
+    <col min="2" max="2" width="5.625" customWidth="1"/>
+    <col min="3" max="3" width="36.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.625" customWidth="1"/>
+    <col min="5" max="7" width="20.125" customWidth="1"/>
+    <col min="8" max="8" width="5.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:8" ht="15" thickBot="1">
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8">
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
@@ -751,7 +774,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:8" ht="18">
       <c r="B3" s="6" t="s">
         <v>8</v>
       </c>
@@ -768,7 +791,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8">
       <c r="B4" s="6" t="s">
         <v>8</v>
       </c>
@@ -781,7 +804,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8">
       <c r="B5" s="6" t="s">
         <v>8</v>
       </c>
@@ -794,7 +817,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8">
       <c r="B6" s="6" t="s">
         <v>8</v>
       </c>
@@ -807,24 +830,24 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8">
       <c r="B7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
       <c r="H7" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8">
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
@@ -837,7 +860,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8">
       <c r="B9" s="6" t="s">
         <v>8</v>
       </c>
@@ -850,24 +873,24 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8">
       <c r="B10" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
       <c r="H10" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8">
       <c r="B11" s="6" t="s">
         <v>8</v>
       </c>
@@ -880,7 +903,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8">
       <c r="B12" s="6" t="s">
         <v>8</v>
       </c>
@@ -893,7 +916,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8">
       <c r="B13" s="6" t="s">
         <v>8</v>
       </c>
@@ -908,35 +931,35 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8">
       <c r="B14" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="17"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="16"/>
       <c r="H14" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8">
       <c r="B15" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="20"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="19"/>
       <c r="H15" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8">
       <c r="B16" s="6" t="s">
         <v>8</v>
       </c>
@@ -949,7 +972,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8">
       <c r="B17" s="6" t="s">
         <v>8</v>
       </c>
@@ -964,35 +987,35 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8">
       <c r="B18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23"/>
+      <c r="C18" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="22"/>
       <c r="H18" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:8" ht="29.25" customHeight="1">
       <c r="B19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="26"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="25"/>
       <c r="H19" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8">
       <c r="B20" s="6" t="s">
         <v>8</v>
       </c>
@@ -1005,7 +1028,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8">
       <c r="B21" s="6" t="s">
         <v>8</v>
       </c>
@@ -1020,35 +1043,35 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:8">
       <c r="B22" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="23"/>
+      <c r="C22" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="32"/>
       <c r="H22" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8">
       <c r="B23" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="26"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="35"/>
       <c r="H23" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:8">
       <c r="B24" s="6" t="s">
         <v>8</v>
       </c>
@@ -1061,7 +1084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8">
       <c r="B25" s="6" t="s">
         <v>8</v>
       </c>
@@ -1084,22 +1107,22 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8">
       <c r="B26" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="29"/>
+      <c r="C26" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="28"/>
       <c r="H26" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="15" thickBot="1">
       <c r="B27" s="11" t="s">
         <v>8</v>
       </c>
@@ -1122,7 +1145,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:8">
       <c r="H28" s="1"/>
     </row>
   </sheetData>

</xml_diff>